<commit_message>
feat: add LLM response cache for Gemini provider
</commit_message>
<xml_diff>
--- a/sample_outputs/QA_COPILOT_Report.xlsx
+++ b/sample_outputs/QA_COPILOT_Report.xlsx
@@ -23,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -33,7 +33,7 @@
     </font>
     <font>
       <b val="1"/>
-      <sz val="18"/>
+      <sz val="20"/>
     </font>
     <font>
       <i val="1"/>
@@ -45,6 +45,10 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="14"/>
     </font>
   </fonts>
   <fills count="3">
@@ -78,7 +82,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -91,6 +95,10 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -456,11 +464,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="31" customWidth="1" min="1" max="1"/>
-    <col width="23" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -477,85 +485,99 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Version</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>v1.7.0</t>
-        </is>
-      </c>
-    </row>
+    <row r="3"/>
     <row r="4"/>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+    <row r="5"/>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>Metric</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>Overall Quality Score</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="n">
-        <v>47</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Quality Verdict</t>
+          <t>Generated On</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>NEEDS CLARIFICATION</t>
+          <t>14-Jul-2026 12:54</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Ambiguity Level</t>
+          <t>Version</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>v1.7.0</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Overall Risk Level</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
+          <t>Overall Quality Score</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>55</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
+          <t>Quality Verdict</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>NEEDS CLARIFICATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Ambiguity Level</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Overall Risk Level</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
           <t>Acceptance Criteria</t>
         </is>
       </c>
-      <c r="B10" s="5" t="n">
-        <v>8</v>
+      <c r="B13" s="5" t="n">
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -573,9 +595,61 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="454" customWidth="1" min="1" max="1"/>
+    <col width="5" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>QA COPILOT</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Requirement Analysis Report</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>REQUIREMENT SUMMARY</t>
+        </is>
+      </c>
+    </row>
+    <row r="5"/>
+    <row r="6" ht="180" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>The system allows customers to transfer money between their own bank accounts by selecting source and destination accounts. Transfers are limited by the available balance, and amounts over ₹1,00,000 require OTP verification. Successful transfers generate a transaction reference number, while failed transfers ensure account balances remain unchanged. The system must complete transfers within 3 seconds, and all transactions are recorded for audit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7"/>
+    <row r="8"/>
+    <row r="9"/>
+    <row r="10"/>
+    <row r="11"/>
+    <row r="12"/>
+    <row r="13"/>
+    <row r="14"/>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A6:B18"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A1:B1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>